<commit_message>
Add prompts and clues, flip columns for IDs to match data
</commit_message>
<xml_diff>
--- a/docs/card_game.xlsx
+++ b/docs/card_game.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WZB Dropbox\Macartan Humphreys\5_github\ci\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ci\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AC5D98F5-5997-4AE9-AD5D-D77AB5B4E520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69399F85-25EF-4922-B0FC-8CF4BC2AA431}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{F65E0536-16B4-41F9-AF18-98A2B651674E}"/>
   </bookViews>
@@ -20,14 +20,13 @@
     <sheet name="formatted d" sheetId="5" r:id="rId5"/>
     <sheet name="formatted e" sheetId="4" r:id="rId6"/>
     <sheet name="formatted f" sheetId="8" r:id="rId7"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="152">
   <si>
     <t>ID</t>
   </si>
@@ -420,6 +419,69 @@
   </si>
   <si>
     <t>ID: F20</t>
+  </si>
+  <si>
+    <t>Clue: -1</t>
+  </si>
+  <si>
+    <t>Clue: -9</t>
+  </si>
+  <si>
+    <t>Clue: 3</t>
+  </si>
+  <si>
+    <t>Clue: 1</t>
+  </si>
+  <si>
+    <t>Clue: -19</t>
+  </si>
+  <si>
+    <t>Clue: 5</t>
+  </si>
+  <si>
+    <t>Clue: 9</t>
+  </si>
+  <si>
+    <t>Clue: 15</t>
+  </si>
+  <si>
+    <t>Clue: -17</t>
+  </si>
+  <si>
+    <t>Clue: -7</t>
+  </si>
+  <si>
+    <t>Clue: 19</t>
+  </si>
+  <si>
+    <t>Clue: -3</t>
+  </si>
+  <si>
+    <t>Clue: 17</t>
+  </si>
+  <si>
+    <t>Clue: -15</t>
+  </si>
+  <si>
+    <t>Clue: 7</t>
+  </si>
+  <si>
+    <t>Clue: 13</t>
+  </si>
+  <si>
+    <t>Clue: -11</t>
+  </si>
+  <si>
+    <t>Clue: 11</t>
+  </si>
+  <si>
+    <t>Clue: -5</t>
+  </si>
+  <si>
+    <t>Clue: -13</t>
+  </si>
+  <si>
+    <t>Choose the left number.</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1114,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1094,50 +1156,68 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1153,7 +1233,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1450,7 +1530,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F356975-8D7A-4B99-8033-B9B7195E3A72}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -2192,7 +2272,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{415304C7-E0D9-41E7-AB48-C70F7B54CADF}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -2225,13 +2305,13 @@
         <v>1</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -2251,13 +2331,13 @@
         <v>12</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2277,13 +2357,13 @@
         <v>2</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2303,13 +2383,13 @@
         <v>18</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -2329,13 +2409,13 @@
         <v>7</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="10"/>
+        <v>25</v>
+      </c>
+      <c r="F6" s="11"/>
       <c r="G6" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="11"/>
+        <v>15</v>
+      </c>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -2355,13 +2435,13 @@
         <v>4</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2381,13 +2461,13 @@
         <v>16</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2407,13 +2487,13 @@
         <v>5</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -2433,13 +2513,13 @@
         <v>13</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -2459,16 +2539,16 @@
         <v>17</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13"/>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2476,7 +2556,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C9FE9D9-EBC5-4C63-B082-407BA7B855C8}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -2509,13 +2589,13 @@
         <v>20</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -2535,13 +2615,13 @@
         <v>9</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2561,13 +2641,13 @@
         <v>19</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2587,13 +2667,13 @@
         <v>3</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -2613,13 +2693,13 @@
         <v>14</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -2639,13 +2719,13 @@
         <v>17</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2665,13 +2745,13 @@
         <v>5</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2691,13 +2771,13 @@
         <v>16</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -2717,13 +2797,13 @@
         <v>8</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -2743,13 +2823,13 @@
         <v>4</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2760,7 +2840,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79154101-B362-4C4B-A855-7009D6A38063}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -2793,13 +2873,17 @@
         <v>25</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="7" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -2819,13 +2903,17 @@
         <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="10" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2845,13 +2933,17 @@
         <v>24</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="10" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2871,13 +2963,17 @@
         <v>8</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="10" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -2897,13 +2993,17 @@
         <v>19</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="10" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -2923,13 +3023,17 @@
         <v>22</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2949,13 +3053,17 @@
         <v>10</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2975,13 +3083,17 @@
         <v>21</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -3001,13 +3113,17 @@
         <v>13</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -3027,13 +3143,17 @@
         <v>9</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13" t="s">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3044,7 +3164,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EBE077F-1651-4F9E-8A52-7581F4727435}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -3077,13 +3197,17 @@
         <v>44</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="7" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -3103,13 +3227,17 @@
         <v>11</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="10" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -3129,13 +3257,17 @@
         <v>41</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="10" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3155,13 +3287,17 @@
         <v>-7</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="10" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -3181,13 +3317,17 @@
         <v>26</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="10" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -3207,13 +3347,17 @@
         <v>35</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -3233,13 +3377,17 @@
         <v>-1</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -3259,13 +3407,17 @@
         <v>32</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -3285,13 +3437,17 @@
         <v>8</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -3311,13 +3467,17 @@
         <v>-4</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13" t="s">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3328,7 +3488,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAC24E2A-1B61-4558-9E05-2222A8A839E0}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -3361,13 +3521,13 @@
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -3387,13 +3547,13 @@
         <v>15</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -3413,13 +3573,13 @@
         <v>15</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3439,13 +3599,13 @@
         <v>15</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -3465,13 +3625,13 @@
         <v>15</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -3491,13 +3651,13 @@
         <v>15</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="11"/>
+      <c r="G7" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -3517,13 +3677,13 @@
         <v>15</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -3543,13 +3703,13 @@
         <v>15</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -3569,13 +3729,13 @@
         <v>15</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -3595,13 +3755,13 @@
         <v>15</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3612,7 +3772,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD2E2A45-D6AC-46B2-948B-360D0376C98D}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="25" customWidth="1"/>
   </cols>
@@ -3645,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="18"/>
+      <c r="G2" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="H2" s="8"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -3671,13 +3831,17 @@
         <v>29</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="19" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -3697,13 +3861,15 @@
         <v>9</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3723,13 +3889,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="19"/>
+      <c r="G5" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="19" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -3749,13 +3917,15 @@
         <v>19</v>
       </c>
       <c r="E6" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -3775,13 +3945,15 @@
         <v>13</v>
       </c>
       <c r="E7" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -3801,13 +3973,15 @@
         <v>37</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="19"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -3827,13 +4001,15 @@
         <v>15</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="19"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -3853,13 +4029,15 @@
         <v>31</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="H10" s="11"/>
+      <c r="H10" s="19"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -3879,25 +4057,18 @@
         <v>5</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="20"/>
+      <c r="G11" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="H11" s="14"/>
+      <c r="H11" s="20" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{827E10FA-3500-44E1-8826-09971D34C236}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Printed version of card game
Added prompts and clues to remaining groups
Some layout changes
</commit_message>
<xml_diff>
--- a/docs/card_game.xlsx
+++ b/docs/card_game.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\ci\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69399F85-25EF-4922-B0FC-8CF4BC2AA431}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87DC9B7-E38B-48CC-AEA3-2AE43EC31CA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{F65E0536-16B4-41F9-AF18-98A2B651674E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24120" windowHeight="9525" activeTab="6" xr2:uid="{F65E0536-16B4-41F9-AF18-98A2B651674E}"/>
   </bookViews>
   <sheets>
     <sheet name="card_game" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="152">
   <si>
     <t>ID</t>
   </si>
@@ -1114,7 +1114,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1129,31 +1129,13 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1173,6 +1155,15 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2304,14 +2295,14 @@
         <f>card_game!F12</f>
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="6" t="s">
+      <c r="F2" s="12"/>
+      <c r="G2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -2330,14 +2321,18 @@
         <f>card_game!F13</f>
         <v>12</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="9" t="s">
+      <c r="F3" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="H3" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2356,14 +2351,16 @@
         <f>card_game!F14</f>
         <v>2</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="9" t="s">
+      <c r="F4" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2382,14 +2379,16 @@
         <f>card_game!F15</f>
         <v>18</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="13"/>
+      <c r="G5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -2408,14 +2407,16 @@
         <f>card_game!F16</f>
         <v>7</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="10"/>
+      <c r="F6" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -2434,14 +2435,16 @@
         <f>card_game!F17</f>
         <v>4</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2460,14 +2463,16 @@
         <f>card_game!F18</f>
         <v>16</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2486,14 +2491,16 @@
         <f>card_game!F19</f>
         <v>5</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G9" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="10"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -2512,14 +2519,16 @@
         <f>card_game!F20</f>
         <v>13</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="9" t="s">
+      <c r="F10" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="10"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -2538,17 +2547,19 @@
         <f>card_game!F21</f>
         <v>17</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>30</v>
       </c>
       <c r="F11" s="14"/>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="13"/>
+      <c r="H11" s="14" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2588,14 +2599,14 @@
         <f>card_game!G12</f>
         <v>20</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="6" t="s">
+      <c r="F2" s="12"/>
+      <c r="G2" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -2614,14 +2625,18 @@
         <f>card_game!G13</f>
         <v>9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="9" t="s">
+      <c r="F3" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="H3" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2640,14 +2655,16 @@
         <f>card_game!G14</f>
         <v>19</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="9" t="s">
+      <c r="F4" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2666,14 +2683,16 @@
         <f>card_game!G15</f>
         <v>3</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="13"/>
+      <c r="G5" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -2692,14 +2711,16 @@
         <f>card_game!G16</f>
         <v>14</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="9" t="s">
+      <c r="F6" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G6" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="10"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -2718,14 +2739,16 @@
         <f>card_game!G17</f>
         <v>17</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2744,14 +2767,16 @@
         <f>card_game!G18</f>
         <v>5</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2770,14 +2795,16 @@
         <f>card_game!G19</f>
         <v>16</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G9" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="H9" s="10"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -2796,14 +2823,16 @@
         <f>card_game!G20</f>
         <v>8</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="9" t="s">
+      <c r="F10" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="H10" s="10"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -2822,17 +2851,19 @@
         <f>card_game!G21</f>
         <v>4</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="14"/>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="13"/>
+      <c r="H11" s="14" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2872,16 +2903,16 @@
         <f>card_game!H12</f>
         <v>25</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>131</v>
       </c>
     </row>
@@ -2902,16 +2933,16 @@
         <f>card_game!H13</f>
         <v>14</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="7" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2932,16 +2963,16 @@
         <f>card_game!H14</f>
         <v>24</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="7" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2962,16 +2993,16 @@
         <f>card_game!H15</f>
         <v>8</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="7" t="s">
         <v>134</v>
       </c>
     </row>
@@ -2992,16 +3023,16 @@
         <f>card_game!H16</f>
         <v>19</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="7" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3022,16 +3053,16 @@
         <f>card_game!H17</f>
         <v>22</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="7" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3052,16 +3083,16 @@
         <f>card_game!H18</f>
         <v>10</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="7" t="s">
         <v>137</v>
       </c>
     </row>
@@ -3082,16 +3113,16 @@
         <f>card_game!H19</f>
         <v>21</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="7" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3112,16 +3143,16 @@
         <f>card_game!H20</f>
         <v>13</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="7" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3142,21 +3173,21 @@
         <f>card_game!H21</f>
         <v>9</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="8" t="s">
         <v>140</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -3196,16 +3227,16 @@
         <f>card_game!I12</f>
         <v>44</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3226,16 +3257,16 @@
         <f>card_game!I13</f>
         <v>11</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="7" t="s">
         <v>132</v>
       </c>
     </row>
@@ -3256,16 +3287,16 @@
         <f>card_game!I14</f>
         <v>41</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="7" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3286,16 +3317,16 @@
         <f>card_game!I15</f>
         <v>-7</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="7" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3316,16 +3347,16 @@
         <f>card_game!I16</f>
         <v>26</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="7" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3346,16 +3377,16 @@
         <f>card_game!I17</f>
         <v>35</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="7" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3376,16 +3407,16 @@
         <f>card_game!I18</f>
         <v>-1</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="7" t="s">
         <v>137</v>
       </c>
     </row>
@@ -3406,16 +3437,16 @@
         <f>card_game!I19</f>
         <v>32</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="7" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3436,16 +3467,16 @@
         <f>card_game!I20</f>
         <v>8</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="7" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3466,21 +3497,21 @@
         <f>card_game!I21</f>
         <v>-4</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="8" t="s">
         <v>140</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -3520,14 +3551,18 @@
         <f>card_game!J12</f>
         <v>15</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="6" t="s">
+      <c r="F2" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="G2" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="H2" s="7"/>
+      <c r="H2" s="6" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -3546,14 +3581,18 @@
         <f>card_game!J13</f>
         <v>15</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="9" t="s">
+      <c r="F3" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="H3" s="7" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -3572,14 +3611,18 @@
         <f>card_game!J14</f>
         <v>15</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="9" t="s">
+      <c r="F4" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="7" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3598,14 +3641,18 @@
         <f>card_game!J15</f>
         <v>15</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="7" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="6" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -3624,14 +3671,18 @@
         <f>card_game!J16</f>
         <v>15</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="9" t="s">
+      <c r="F6" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="H6" s="10"/>
+      <c r="H6" s="7" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -3650,14 +3701,18 @@
         <f>card_game!J17</f>
         <v>15</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="7" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -3676,14 +3731,18 @@
         <f>card_game!J18</f>
         <v>15</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="7" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -3702,14 +3761,18 @@
         <f>card_game!J19</f>
         <v>15</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="H9" s="10"/>
+      <c r="H9" s="7" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -3728,14 +3791,18 @@
         <f>card_game!J20</f>
         <v>15</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="9" t="s">
+      <c r="F10" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="10"/>
+      <c r="H10" s="7" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -3754,17 +3821,21 @@
         <f>card_game!J21</f>
         <v>15</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="12" t="s">
+      <c r="F11" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="H11" s="13"/>
+      <c r="H11" s="8" t="s">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
@@ -3804,14 +3875,14 @@
         <f>card_game!K12</f>
         <v>5</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="6" t="s">
+      <c r="F2" s="12"/>
+      <c r="G2" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="H2" s="18"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -3830,16 +3901,16 @@
         <f>card_game!K13</f>
         <v>29</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="13" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3860,16 +3931,16 @@
         <f>card_game!K14</f>
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="19"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3888,14 +3959,14 @@
         <f>card_game!K15</f>
         <v>5</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="19"/>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="13"/>
+      <c r="G5" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="13" t="s">
         <v>151</v>
       </c>
     </row>
@@ -3916,16 +3987,16 @@
         <f>card_game!K16</f>
         <v>19</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -3944,16 +4015,16 @@
         <f>card_game!K17</f>
         <v>13</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="19"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -3972,16 +4043,16 @@
         <f>card_game!K18</f>
         <v>37</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="H8" s="19"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -4000,16 +4071,16 @@
         <f>card_game!K19</f>
         <v>15</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="H9" s="19"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -4028,16 +4099,16 @@
         <f>card_game!K20</f>
         <v>31</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="H10" s="19"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:8" s="3" customFormat="1" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -4056,19 +4127,19 @@
         <f>card_game!K21</f>
         <v>5</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="20"/>
-      <c r="G11" s="12" t="s">
+      <c r="F11" s="14"/>
+      <c r="G11" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="14" t="s">
         <v>151</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>